<commit_message>
formatting task work completed in this commit
</commit_message>
<xml_diff>
--- a/Data Entry.xlsx
+++ b/Data Entry.xlsx
@@ -5,17 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASDC11\Desktop\Github-Smit\Data_Analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASDC11\Desktop\Smit\Data_Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EAF733-BA4B-46B8-B5E3-AE13557572EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FB305E-67B0-4E67-9BAF-D2BA7804B9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{76D07AF9-5284-495A-A2FD-6FB15EBF7EF8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{76D07AF9-5284-495A-A2FD-6FB15EBF7EF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Entry" sheetId="1" r:id="rId1"/>
     <sheet name="Split" sheetId="2" r:id="rId2"/>
     <sheet name="Task3" sheetId="3" r:id="rId3"/>
+    <sheet name="Employee Sheet" sheetId="4" r:id="rId4"/>
+    <sheet name="Sales Report" sheetId="5" r:id="rId5"/>
+    <sheet name="Student Marks Sheet" sheetId="6" r:id="rId6"/>
+    <sheet name="Sales Summary" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="212">
   <si>
     <t>Name</t>
   </si>
@@ -310,17 +314,391 @@
   </si>
   <si>
     <t>com</t>
+  </si>
+  <si>
+    <t>24/01/2026</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Joining Date</t>
+  </si>
+  <si>
+    <t>E101</t>
+  </si>
+  <si>
+    <t>Amit Sharma</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>E102</t>
+  </si>
+  <si>
+    <t>Neha Verma</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>E103</t>
+  </si>
+  <si>
+    <t>Rahul Mehta</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>E104</t>
+  </si>
+  <si>
+    <t>Pooja Singh</t>
+  </si>
+  <si>
+    <t>E105</t>
+  </si>
+  <si>
+    <t>Ankit Patel</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>E106</t>
+  </si>
+  <si>
+    <t>E107</t>
+  </si>
+  <si>
+    <t>E108</t>
+  </si>
+  <si>
+    <t>E109</t>
+  </si>
+  <si>
+    <t>E110</t>
+  </si>
+  <si>
+    <t>E111</t>
+  </si>
+  <si>
+    <t>E112</t>
+  </si>
+  <si>
+    <t>E113</t>
+  </si>
+  <si>
+    <t>E114</t>
+  </si>
+  <si>
+    <t>E115</t>
+  </si>
+  <si>
+    <t>Darshan Sarvaiya</t>
+  </si>
+  <si>
+    <t>Vaidik Limbachiya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dhairy gehlot </t>
+  </si>
+  <si>
+    <t>E116</t>
+  </si>
+  <si>
+    <t>E117</t>
+  </si>
+  <si>
+    <t>E118</t>
+  </si>
+  <si>
+    <t>E119</t>
+  </si>
+  <si>
+    <t>E120</t>
+  </si>
+  <si>
+    <t>Shivam Thakar</t>
+  </si>
+  <si>
+    <t>Vishv Patel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nirmal Lohar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aashita Prajapati </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhavy Maniyar </t>
+  </si>
+  <si>
+    <t>Drasti Pithva</t>
+  </si>
+  <si>
+    <t>Yashvi Joshi</t>
+  </si>
+  <si>
+    <t>Keyuri Patel</t>
+  </si>
+  <si>
+    <t>Isha Makvana</t>
+  </si>
+  <si>
+    <t>Format header row (Bold, Color)
+Salary → Currency (₹)
+Date → Date format
+Apply borders and auto-fit columns</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Sales Amount</t>
+  </si>
+  <si>
+    <t>Salesperson</t>
+  </si>
+  <si>
+    <t>Laptop Dell Inspiron 15</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>Ramesh</t>
+  </si>
+  <si>
+    <t>HP Wireless Mouse</t>
+  </si>
+  <si>
+    <t>West</t>
+  </si>
+  <si>
+    <t>Sneha</t>
+  </si>
+  <si>
+    <t>Samsung 24-inch Monitor</t>
+  </si>
+  <si>
+    <t>East</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Lenovo ThinkPad E14 Laptop</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Kavita</t>
+  </si>
+  <si>
+    <t>Add title Monthly Sales Report
+Merge &amp; center title
+Wrap text for product names
+Currency format for sales</t>
+  </si>
+  <si>
+    <t>Task 2</t>
+  </si>
+  <si>
+    <t>Monthly Sales Report</t>
+  </si>
+  <si>
+    <t>Laptop Dell Inspiron 16</t>
+  </si>
+  <si>
+    <t>Laptop Dell Inspiron 17</t>
+  </si>
+  <si>
+    <t>Laptop Dell Inspiron 18</t>
+  </si>
+  <si>
+    <t>Laptop Dell Inspiron 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task 3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student Marks Sheet </t>
+  </si>
+  <si>
+    <t>Roll No</t>
+  </si>
+  <si>
+    <t>Student Name</t>
+  </si>
+  <si>
+    <t>Maths</t>
+  </si>
+  <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>Aakash</t>
+  </si>
+  <si>
+    <t>Bhavya</t>
+  </si>
+  <si>
+    <t>Chirag</t>
+  </si>
+  <si>
+    <t>Divya</t>
+  </si>
+  <si>
+    <t>Esha</t>
+  </si>
+  <si>
+    <t>Isha</t>
+  </si>
+  <si>
+    <t>Darshan</t>
+  </si>
+  <si>
+    <t>Vaidik</t>
+  </si>
+  <si>
+    <t>Keyur</t>
+  </si>
+  <si>
+    <t>Vishv</t>
+  </si>
+  <si>
+    <t>Riddhi</t>
+  </si>
+  <si>
+    <t>Yashvi</t>
+  </si>
+  <si>
+    <t>Keyuri</t>
+  </si>
+  <si>
+    <t>Drasti</t>
+  </si>
+  <si>
+    <t>Meet</t>
+  </si>
+  <si>
+    <t>Sumit</t>
+  </si>
+  <si>
+    <t>Calculate Percentage
+Format percentage column
+Apply cell styles to headers</t>
+  </si>
+  <si>
+    <t>Task 4</t>
+  </si>
+  <si>
+    <t>Invoice No</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>INV001</t>
+  </si>
+  <si>
+    <t>INV002</t>
+  </si>
+  <si>
+    <t>INV003</t>
+  </si>
+  <si>
+    <t>INV004</t>
+  </si>
+  <si>
+    <t>INV005</t>
+  </si>
+  <si>
+    <t>Calculate Total Sales
+Find Average Sales
+Identify Highest &amp; Lowest Sale</t>
+  </si>
+  <si>
+    <t>INV006</t>
+  </si>
+  <si>
+    <t>INV007</t>
+  </si>
+  <si>
+    <t>INV008</t>
+  </si>
+  <si>
+    <t>INV009</t>
+  </si>
+  <si>
+    <t>INV010</t>
+  </si>
+  <si>
+    <t>INV011</t>
+  </si>
+  <si>
+    <t>INV012</t>
+  </si>
+  <si>
+    <t>INV013</t>
+  </si>
+  <si>
+    <t>INV014</t>
+  </si>
+  <si>
+    <t>INV015</t>
+  </si>
+  <si>
+    <t>INV016</t>
+  </si>
+  <si>
+    <t>INV017</t>
+  </si>
+  <si>
+    <t>INV018</t>
+  </si>
+  <si>
+    <t>INV019</t>
+  </si>
+  <si>
+    <t>INV020</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>AVG SALES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="[$₹-4009]\ #,##0.0"/>
-    <numFmt numFmtId="166" formatCode="[$₹-4009]\ #,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="[$₹-4009]\ #,##0.0"/>
+    <numFmt numFmtId="165" formatCode="[$₹-4009]\ #,##0.00"/>
+    <numFmt numFmtId="175" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,8 +759,118 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFF0F6FC"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -425,8 +913,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -462,12 +968,133 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF3D444D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF3D444D"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF3D444D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF3D444D"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -484,12 +1111,12 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -502,24 +1129,1216 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="14" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="21" fillId="10" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="21" fillId="10" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="[$₹-4009]\ #,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="[$₹-4009]\ #,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="[$₹-4009]\ #,##0.00"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="0"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FF3D444D"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF3D444D"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF3D444D"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF3D444D"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -530,6 +2349,65 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A48F8CFE-A386-463A-B6B5-64545F3BD8E5}" name="Table1" displayName="Table1" ref="B4:F24" totalsRowShown="0" headerRowDxfId="31" dataDxfId="32" headerRowBorderDxfId="37" tableBorderDxfId="38" totalsRowBorderDxfId="36">
+  <autoFilter ref="B4:F24" xr:uid="{A48F8CFE-A386-463A-B6B5-64545F3BD8E5}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{DEE9CFDA-EB1B-4BC7-B118-3FDD03FE3344}" name="Employee ID" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{7FAF82BA-1318-4192-A77F-353BC51342E6}" name="Name" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{AD4B3451-A8F2-4FA4-BA14-410A37F18CC8}" name="Department" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{9749CDEE-F7F9-4953-97A2-4EB0109A465E}" name="Salary" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{86C8D64E-B733-4168-B2BB-AA9E25799793}" name="Joining Date" dataDxfId="29"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{03BD9F59-6B96-4714-8806-ADC5EB8D228C}" name="Table3" displayName="Table3" ref="B5:E25" totalsRowShown="0" headerRowDxfId="25" dataDxfId="20" headerRowBorderDxfId="27" tableBorderDxfId="28" totalsRowBorderDxfId="26">
+  <autoFilter ref="B5:E25" xr:uid="{03BD9F59-6B96-4714-8806-ADC5EB8D228C}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{F80BE902-6D79-41EE-BF44-E2DCB650DD7A}" name="Product Name" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{6E1662D4-B433-41AF-A382-C389F48DDD5C}" name="Region" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{E8D45F3F-86DC-4995-9BE9-7C5C6A0327EE}" name="Sales Amount" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{46186AFC-E5EE-483F-859D-8BE002E1B6FB}" name="Salesperson" dataDxfId="21"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{14C88445-DA0B-40F4-B89C-1259878389AA}" name="Table4" displayName="Table4" ref="B5:H25" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="18" tableBorderDxfId="19" totalsRowBorderDxfId="17">
+  <autoFilter ref="B5:H25" xr:uid="{14C88445-DA0B-40F4-B89C-1259878389AA}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{DAA8C6D4-C273-486F-8761-547FD319997D}" name="Roll No" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{9FE05849-077D-4789-9F2B-007F0E23D181}" name="Student Name" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{B08ADC76-1D8C-432A-B776-038B27EC389F}" name="Maths" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{AE8AA3CF-2328-49F6-B641-65F032751A82}" name="Science" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0581BFB5-AB7E-4E88-8F0C-B2D8D1EA780A}" name="English" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{FFAC8AC2-B6E2-41FC-9EC8-F572F080187A}" name="Total" dataDxfId="9">
+      <calculatedColumnFormula>SUM(Table4[[#This Row],[Maths]:[English]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{F955AED9-4EBA-4EA3-A2B1-421664FE37C8}" name="Percentage" dataDxfId="8" dataCellStyle="Percent">
+      <calculatedColumnFormula>Table4[[#This Row],[Total]]/300</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{09B25C05-6FB7-439C-BE1F-14B0F3A6D2FB}" name="Table5" displayName="Table5" ref="B3:D23" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="B3:D23" xr:uid="{09B25C05-6FB7-439C-BE1F-14B0F3A6D2FB}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{AAEF1950-EC49-4D17-BBA1-BCE6FF516076}" name="Invoice No" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{DD3502FE-8459-422D-91BE-7AEF89BC1984}" name="Date" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{339D8814-3169-4D99-852A-AB0B1ADF9523}" name="Sales Amount" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2026,4 +3904,1756 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{123E0D17-87A5-44E4-851F-782BCD7F7032}">
+  <dimension ref="B1:T24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="32" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:20" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B1" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+    </row>
+    <row r="2" spans="2:20" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="M3" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="29"/>
+    </row>
+    <row r="4" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="29"/>
+      <c r="S4" s="29"/>
+      <c r="T4" s="29"/>
+    </row>
+    <row r="5" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="24">
+        <v>32000</v>
+      </c>
+      <c r="F5" s="31">
+        <v>44573</v>
+      </c>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="29"/>
+      <c r="T5" s="29"/>
+    </row>
+    <row r="6" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" s="24">
+        <v>45000</v>
+      </c>
+      <c r="F6" s="32">
+        <v>44260</v>
+      </c>
+      <c r="M6" s="29"/>
+      <c r="N6" s="29"/>
+      <c r="O6" s="29"/>
+      <c r="P6" s="29"/>
+      <c r="Q6" s="29"/>
+      <c r="R6" s="29"/>
+      <c r="S6" s="29"/>
+      <c r="T6" s="29"/>
+    </row>
+    <row r="7" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="24">
+        <v>38000</v>
+      </c>
+      <c r="F7" s="32">
+        <v>44030</v>
+      </c>
+      <c r="M7" s="29"/>
+      <c r="N7" s="29"/>
+      <c r="O7" s="29"/>
+      <c r="P7" s="29"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="29"/>
+      <c r="S7" s="29"/>
+      <c r="T7" s="29"/>
+    </row>
+    <row r="8" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="24">
+        <v>52000</v>
+      </c>
+      <c r="F8" s="32">
+        <v>43779</v>
+      </c>
+      <c r="M8" s="29"/>
+      <c r="N8" s="29"/>
+      <c r="O8" s="29"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="29"/>
+      <c r="R8" s="29"/>
+      <c r="S8" s="29"/>
+      <c r="T8" s="29"/>
+    </row>
+    <row r="9" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B9" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" s="25">
+        <v>30000</v>
+      </c>
+      <c r="F9" s="32">
+        <v>45102</v>
+      </c>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
+    </row>
+    <row r="10" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="24">
+        <v>50000</v>
+      </c>
+      <c r="F10" s="31">
+        <v>43565</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E11" s="24">
+        <v>75000</v>
+      </c>
+      <c r="F11" s="32">
+        <v>43254</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" ht="41.25" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E12" s="24">
+        <v>60000</v>
+      </c>
+      <c r="F12" s="32">
+        <v>44395</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="24">
+        <v>25000</v>
+      </c>
+      <c r="F13" s="32">
+        <v>43809</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" s="24">
+        <v>30000</v>
+      </c>
+      <c r="F14" s="32">
+        <v>45468</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" s="24">
+        <v>28000</v>
+      </c>
+      <c r="F15" s="31">
+        <v>42529</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="24">
+        <v>35000</v>
+      </c>
+      <c r="F16" s="32">
+        <v>42186</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="24">
+        <v>40000</v>
+      </c>
+      <c r="F17" s="32">
+        <v>44760</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="24">
+        <v>60000</v>
+      </c>
+      <c r="F18" s="32">
+        <v>43751</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B19" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="24">
+        <v>35000</v>
+      </c>
+      <c r="F19" s="32">
+        <v>45833</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B20" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="E20" s="24">
+        <v>15000</v>
+      </c>
+      <c r="F20" s="31">
+        <v>41523</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="20" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" s="24">
+        <v>25000</v>
+      </c>
+      <c r="F21" s="32">
+        <v>40827</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B22" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="24">
+        <v>45000</v>
+      </c>
+      <c r="F22" s="32">
+        <v>45125</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B23" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="24">
+        <v>55000</v>
+      </c>
+      <c r="F23" s="32">
+        <v>43752</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="21" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="24">
+        <v>38000</v>
+      </c>
+      <c r="F24" s="32">
+        <v>46198</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="M3:T9"/>
+  </mergeCells>
+  <phoneticPr fontId="15" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2114BF9F-BF2F-4D17-963C-1A035D36B8BD}">
+  <dimension ref="B1:U25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:21" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B1" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+    </row>
+    <row r="3" spans="2:21" ht="21" x14ac:dyDescent="0.35">
+      <c r="B3" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+    </row>
+    <row r="5" spans="2:21" s="39" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="40" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="O5" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="27"/>
+      <c r="T5" s="27"/>
+      <c r="U5" s="27"/>
+    </row>
+    <row r="6" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="44" t="s">
+        <v>142</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="46">
+        <v>45000</v>
+      </c>
+      <c r="E6" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+      <c r="S6" s="27"/>
+      <c r="T6" s="27"/>
+      <c r="U6" s="27"/>
+    </row>
+    <row r="7" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="D7" s="46">
+        <v>1200</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>147</v>
+      </c>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="27"/>
+      <c r="S7" s="27"/>
+      <c r="T7" s="27"/>
+      <c r="U7" s="27"/>
+    </row>
+    <row r="8" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="46">
+        <v>18000</v>
+      </c>
+      <c r="E8" s="47" t="s">
+        <v>150</v>
+      </c>
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="Q8" s="27"/>
+      <c r="R8" s="27"/>
+      <c r="S8" s="27"/>
+      <c r="T8" s="27"/>
+      <c r="U8" s="27"/>
+    </row>
+    <row r="9" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D9" s="50">
+        <v>62000</v>
+      </c>
+      <c r="E9" s="51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="44" t="s">
+        <v>157</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D10" s="46">
+        <v>48500</v>
+      </c>
+      <c r="E10" s="47" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11" s="46">
+        <v>55280</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D12" s="46">
+        <v>62060</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D13" s="50">
+        <v>68840</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="44" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="46">
+        <v>75620</v>
+      </c>
+      <c r="E14" s="47" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="C15" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="46">
+        <v>82400</v>
+      </c>
+      <c r="E15" s="47" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C16" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D16" s="46">
+        <v>89180</v>
+      </c>
+      <c r="E16" s="47" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C17" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D17" s="50">
+        <v>95960</v>
+      </c>
+      <c r="E17" s="51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="44" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D18" s="46">
+        <v>102740</v>
+      </c>
+      <c r="E18" s="47" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="C19" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="D19" s="46">
+        <v>109520</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C20" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D20" s="46">
+        <v>116300</v>
+      </c>
+      <c r="E20" s="47" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D21" s="50">
+        <v>123080</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="C22" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D22" s="46">
+        <v>129860</v>
+      </c>
+      <c r="E22" s="47" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="44" t="s">
+        <v>145</v>
+      </c>
+      <c r="C23" s="45" t="s">
+        <v>146</v>
+      </c>
+      <c r="D23" s="46">
+        <v>136640</v>
+      </c>
+      <c r="E23" s="47" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="44" t="s">
+        <v>148</v>
+      </c>
+      <c r="C24" s="45" t="s">
+        <v>149</v>
+      </c>
+      <c r="D24" s="46">
+        <v>143420</v>
+      </c>
+      <c r="E24" s="47" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="B25" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="C25" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D25" s="50">
+        <v>150200</v>
+      </c>
+      <c r="E25" s="51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="O5:U8"/>
+    <mergeCell ref="B3:E3"/>
+  </mergeCells>
+  <phoneticPr fontId="15" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{021084FD-3C00-4812-83EB-69719DAB5380}">
+  <dimension ref="B1:R25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:18" ht="21" x14ac:dyDescent="0.35">
+      <c r="B1" s="53" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+    </row>
+    <row r="3" spans="2:18" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B3" s="52" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+    </row>
+    <row r="5" spans="2:18" ht="35.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="55" t="s">
+        <v>166</v>
+      </c>
+      <c r="F5" s="55" t="s">
+        <v>167</v>
+      </c>
+      <c r="G5" s="57" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="56" t="s">
+        <v>168</v>
+      </c>
+      <c r="M5" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+    </row>
+    <row r="6" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="58">
+        <v>1</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>169</v>
+      </c>
+      <c r="D6" s="59">
+        <v>78</v>
+      </c>
+      <c r="E6" s="59">
+        <v>82</v>
+      </c>
+      <c r="F6" s="59">
+        <v>74</v>
+      </c>
+      <c r="G6" s="60">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>234</v>
+      </c>
+      <c r="H6" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.78</v>
+      </c>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
+      <c r="R6" s="27"/>
+    </row>
+    <row r="7" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="58">
+        <v>2</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" s="59">
+        <v>65</v>
+      </c>
+      <c r="E7" s="59">
+        <v>70</v>
+      </c>
+      <c r="F7" s="59">
+        <v>68</v>
+      </c>
+      <c r="G7" s="60">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>203</v>
+      </c>
+      <c r="H7" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.67666666666666664</v>
+      </c>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="27"/>
+    </row>
+    <row r="8" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="58">
+        <v>3</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" s="59">
+        <v>90</v>
+      </c>
+      <c r="E8" s="59">
+        <v>88</v>
+      </c>
+      <c r="F8" s="59">
+        <v>92</v>
+      </c>
+      <c r="G8" s="60">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>270</v>
+      </c>
+      <c r="H8" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.9</v>
+      </c>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="Q8" s="27"/>
+      <c r="R8" s="27"/>
+    </row>
+    <row r="9" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="58">
+        <v>4</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" s="59">
+        <v>35</v>
+      </c>
+      <c r="E9" s="59">
+        <v>40</v>
+      </c>
+      <c r="F9" s="59">
+        <v>38</v>
+      </c>
+      <c r="G9" s="60">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>113</v>
+      </c>
+      <c r="H9" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.37666666666666665</v>
+      </c>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="27"/>
+      <c r="R9" s="27"/>
+    </row>
+    <row r="10" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="61">
+        <v>5</v>
+      </c>
+      <c r="C10" s="62" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" s="62">
+        <v>55</v>
+      </c>
+      <c r="E10" s="62">
+        <v>60</v>
+      </c>
+      <c r="F10" s="62">
+        <v>58</v>
+      </c>
+      <c r="G10" s="63">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>173</v>
+      </c>
+      <c r="H10" s="66">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.57666666666666666</v>
+      </c>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="27"/>
+      <c r="Q10" s="27"/>
+      <c r="R10" s="27"/>
+    </row>
+    <row r="11" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="58">
+        <v>6</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="59">
+        <v>82</v>
+      </c>
+      <c r="E11" s="59">
+        <v>44</v>
+      </c>
+      <c r="F11" s="59">
+        <v>78</v>
+      </c>
+      <c r="G11" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>204</v>
+      </c>
+      <c r="H11" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.68</v>
+      </c>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
+      <c r="R11" s="27"/>
+    </row>
+    <row r="12" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="58">
+        <v>7</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>174</v>
+      </c>
+      <c r="D12" s="59">
+        <v>70</v>
+      </c>
+      <c r="E12" s="59">
+        <v>58</v>
+      </c>
+      <c r="F12" s="59">
+        <v>65</v>
+      </c>
+      <c r="G12" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>193</v>
+      </c>
+      <c r="H12" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.64333333333333331</v>
+      </c>
+    </row>
+    <row r="13" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="58">
+        <v>8</v>
+      </c>
+      <c r="C13" s="59" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" s="59">
+        <v>88</v>
+      </c>
+      <c r="E13" s="59">
+        <v>36</v>
+      </c>
+      <c r="F13" s="59">
+        <v>48</v>
+      </c>
+      <c r="G13" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>172</v>
+      </c>
+      <c r="H13" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.57333333333333336</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="58">
+        <v>9</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>176</v>
+      </c>
+      <c r="D14" s="59">
+        <v>40</v>
+      </c>
+      <c r="E14" s="59">
+        <v>88</v>
+      </c>
+      <c r="F14" s="59">
+        <v>37</v>
+      </c>
+      <c r="G14" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>165</v>
+      </c>
+      <c r="H14" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="61">
+        <v>10</v>
+      </c>
+      <c r="C15" s="59" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="62">
+        <v>60</v>
+      </c>
+      <c r="E15" s="59">
+        <v>45</v>
+      </c>
+      <c r="F15" s="59">
+        <v>68</v>
+      </c>
+      <c r="G15" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>173</v>
+      </c>
+      <c r="H15" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.57666666666666666</v>
+      </c>
+    </row>
+    <row r="16" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="58">
+        <v>11</v>
+      </c>
+      <c r="C16" s="59" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="59">
+        <v>74</v>
+      </c>
+      <c r="E16" s="59">
+        <v>70</v>
+      </c>
+      <c r="F16" s="59">
+        <v>59</v>
+      </c>
+      <c r="G16" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>203</v>
+      </c>
+      <c r="H16" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.67666666666666664</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="58">
+        <v>12</v>
+      </c>
+      <c r="C17" s="59" t="s">
+        <v>177</v>
+      </c>
+      <c r="D17" s="59">
+        <v>68</v>
+      </c>
+      <c r="E17" s="59">
+        <v>60</v>
+      </c>
+      <c r="F17" s="59">
+        <v>48</v>
+      </c>
+      <c r="G17" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>176</v>
+      </c>
+      <c r="H17" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.58666666666666667</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="58">
+        <v>13</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>178</v>
+      </c>
+      <c r="D18" s="59">
+        <v>92</v>
+      </c>
+      <c r="E18" s="59">
+        <v>25</v>
+      </c>
+      <c r="F18" s="59">
+        <v>90</v>
+      </c>
+      <c r="G18" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>207</v>
+      </c>
+      <c r="H18" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.69</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="58">
+        <v>14</v>
+      </c>
+      <c r="C19" s="59" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="59">
+        <v>38</v>
+      </c>
+      <c r="E19" s="59">
+        <v>39</v>
+      </c>
+      <c r="F19" s="59">
+        <v>45</v>
+      </c>
+      <c r="G19" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>122</v>
+      </c>
+      <c r="H19" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.40666666666666668</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="61">
+        <v>15</v>
+      </c>
+      <c r="C20" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="D20" s="62">
+        <v>58</v>
+      </c>
+      <c r="E20" s="59">
+        <v>55</v>
+      </c>
+      <c r="F20" s="59">
+        <v>88</v>
+      </c>
+      <c r="G20" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>201</v>
+      </c>
+      <c r="H20" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="58">
+        <v>16</v>
+      </c>
+      <c r="C21" s="59" t="s">
+        <v>180</v>
+      </c>
+      <c r="D21" s="59">
+        <v>78</v>
+      </c>
+      <c r="E21" s="59">
+        <v>84</v>
+      </c>
+      <c r="F21" s="59">
+        <v>90</v>
+      </c>
+      <c r="G21" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>252</v>
+      </c>
+      <c r="H21" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="58">
+        <v>17</v>
+      </c>
+      <c r="C22" s="59" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="59">
+        <v>65</v>
+      </c>
+      <c r="E22" s="59">
+        <v>90</v>
+      </c>
+      <c r="F22" s="59">
+        <v>95</v>
+      </c>
+      <c r="G22" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>250</v>
+      </c>
+      <c r="H22" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="58">
+        <v>18</v>
+      </c>
+      <c r="C23" s="59" t="s">
+        <v>182</v>
+      </c>
+      <c r="D23" s="59">
+        <v>90</v>
+      </c>
+      <c r="E23" s="59">
+        <v>78</v>
+      </c>
+      <c r="F23" s="59">
+        <v>45</v>
+      </c>
+      <c r="G23" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>213</v>
+      </c>
+      <c r="H23" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="58">
+        <v>19</v>
+      </c>
+      <c r="C24" s="59" t="s">
+        <v>183</v>
+      </c>
+      <c r="D24" s="59">
+        <v>35</v>
+      </c>
+      <c r="E24" s="59">
+        <v>63</v>
+      </c>
+      <c r="F24" s="59">
+        <v>76</v>
+      </c>
+      <c r="G24" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>174</v>
+      </c>
+      <c r="H24" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="61">
+        <v>20</v>
+      </c>
+      <c r="C25" s="59" t="s">
+        <v>184</v>
+      </c>
+      <c r="D25" s="62">
+        <v>55</v>
+      </c>
+      <c r="E25" s="59">
+        <v>85</v>
+      </c>
+      <c r="F25" s="59">
+        <v>66</v>
+      </c>
+      <c r="G25" s="64">
+        <f>SUM(Table4[[#This Row],[Maths]:[English]])</f>
+        <v>206</v>
+      </c>
+      <c r="H25" s="65">
+        <f>Table4[[#This Row],[Total]]/300</f>
+        <v>0.68666666666666665</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="M5:R11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBD2495F-ED7B-4EA7-839B-6D2627FA895F}">
+  <dimension ref="B1:P27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:16" ht="21" x14ac:dyDescent="0.35">
+      <c r="B1" s="53" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+    </row>
+    <row r="3" spans="2:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="67" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="D3" s="69" t="s">
+        <v>140</v>
+      </c>
+      <c r="M3" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="N3" s="27"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="27"/>
+    </row>
+    <row r="4" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="34" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="30">
+        <v>45292</v>
+      </c>
+      <c r="D4" s="70">
+        <v>12000</v>
+      </c>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+    </row>
+    <row r="5" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" s="30">
+        <v>45293</v>
+      </c>
+      <c r="D5" s="70">
+        <v>25000</v>
+      </c>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+    </row>
+    <row r="6" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="30">
+        <v>45294</v>
+      </c>
+      <c r="D6" s="70">
+        <v>8000</v>
+      </c>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+    </row>
+    <row r="7" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="34" t="s">
+        <v>192</v>
+      </c>
+      <c r="C7" s="30">
+        <v>45295</v>
+      </c>
+      <c r="D7" s="70">
+        <v>32000</v>
+      </c>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+    </row>
+    <row r="8" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="35" t="s">
+        <v>193</v>
+      </c>
+      <c r="C8" s="30">
+        <v>45296</v>
+      </c>
+      <c r="D8" s="71">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="30">
+        <v>45515</v>
+      </c>
+      <c r="D9" s="70">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" s="30">
+        <v>45513</v>
+      </c>
+      <c r="D10" s="70">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="34" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11" s="30">
+        <v>45584</v>
+      </c>
+      <c r="D11" s="70">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="34" t="s">
+        <v>198</v>
+      </c>
+      <c r="C12" s="30">
+        <v>45447</v>
+      </c>
+      <c r="D12" s="70">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="35" t="s">
+        <v>199</v>
+      </c>
+      <c r="C13" s="30">
+        <v>45648</v>
+      </c>
+      <c r="D13" s="70">
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="34" t="s">
+        <v>200</v>
+      </c>
+      <c r="C14" s="30">
+        <v>45455</v>
+      </c>
+      <c r="D14" s="70">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="34" t="s">
+        <v>201</v>
+      </c>
+      <c r="C15" s="30">
+        <v>45327</v>
+      </c>
+      <c r="D15" s="70">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="C16" s="30">
+        <v>45334</v>
+      </c>
+      <c r="D16" s="70">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="34" t="s">
+        <v>203</v>
+      </c>
+      <c r="C17" s="30">
+        <v>45369</v>
+      </c>
+      <c r="D17" s="70">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="35" t="s">
+        <v>204</v>
+      </c>
+      <c r="C18" s="30">
+        <v>45644</v>
+      </c>
+      <c r="D18" s="70">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="C19" s="30">
+        <v>45509</v>
+      </c>
+      <c r="D19" s="70">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="34" t="s">
+        <v>206</v>
+      </c>
+      <c r="C20" s="30">
+        <v>45595</v>
+      </c>
+      <c r="D20" s="70">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="34" t="s">
+        <v>207</v>
+      </c>
+      <c r="C21" s="30">
+        <v>45458</v>
+      </c>
+      <c r="D21" s="70">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="34" t="s">
+        <v>208</v>
+      </c>
+      <c r="C22" s="30">
+        <v>45509</v>
+      </c>
+      <c r="D22" s="70">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="35" t="s">
+        <v>209</v>
+      </c>
+      <c r="C23" s="30">
+        <v>45625</v>
+      </c>
+      <c r="D23" s="70">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="C25" s="72" t="s">
+        <v>210</v>
+      </c>
+      <c r="D25" s="73">
+        <f>SUM(Table5[Sales Amount])</f>
+        <v>266000</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="C27" s="74" t="s">
+        <v>211</v>
+      </c>
+      <c r="D27" s="75">
+        <f>AVERAGE(Table5[Sales Amount])</f>
+        <v>13300</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="M3:P7"/>
+  </mergeCells>
+  <phoneticPr fontId="15" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>